<commit_message>
updated the user generation function
</commit_message>
<xml_diff>
--- a/final_users.xlsx
+++ b/final_users.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ALNAFE ENOCK CHISATI\Documents\LETS CODE!\DHIS2-SCRIPTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DE8866C-499E-4322-A235-E24F4F688029}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9708C202-B789-4BB3-ABF0-45627DB7E020}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5256" yWindow="2916" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="25">
   <si>
     <t>firstName</t>
   </si>
@@ -82,20 +82,26 @@
     <t>Zalo</t>
   </si>
   <si>
-    <t>Kellingo</t>
-  </si>
-  <si>
     <t>Zaliwo</t>
   </si>
   <si>
     <t>mbewa</t>
+  </si>
+  <si>
+    <t>loy</t>
+  </si>
+  <si>
+    <t>Pellingo</t>
+  </si>
+  <si>
+    <t>m'bewa</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -114,14 +120,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF212934"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -159,11 +157,10 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -174,10 +171,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -480,213 +475,208 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.21875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="20.77734375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="28.88671875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="28.88671875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
       <c r="E1" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="M1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="N1" s="1"/>
+      <c r="L1" s="1"/>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>18</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D2" s="4"/>
-      <c r="F2" s="2">
+        <v>21</v>
+      </c>
+      <c r="D2" s="2">
         <v>123456789</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>11</v>
       </c>
+      <c r="F2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>13</v>
+      </c>
       <c r="H2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I2" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>15</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="M2" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>19</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2" t="s">
+      <c r="B4" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="G4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="I4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="J4" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="M3" s="2" t="s">
+      <c r="K4" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2" t="s">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="F5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="G5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="H5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="K4" s="2" t="s">
+      <c r="I5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="L4" s="2" t="s">
+      <c r="J5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="M4" s="2" t="s">
+      <c r="K5" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2" t="s">
+      <c r="B6" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="F6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="I5" s="3" t="s">
+      <c r="G6" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="J5" s="2" t="s">
+      <c r="H6" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="K5" s="2" t="s">
+      <c r="I6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="L5" s="2" t="s">
+      <c r="J6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="M5" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I6" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>14</v>
-      </c>
       <c r="K6" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="L6" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="M6" s="2" t="s">
         <v>17</v>
       </c>
     </row>

</xml_diff>